<commit_message>
added new template file in data/
</commit_message>
<xml_diff>
--- a/data/template_output.xlsx
+++ b/data/template_output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pfizer-my.sharepoint.com/personal/hoveyo_pfizer_com/Documents/financial-automation-project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_53563E9B681595B0F7239972BC8032DCB2E48D80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7B51FD2-2639-49C3-B5C1-4AC7A0CF7C19}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_53563E9B681595B0F7239972BC8032DCB2E48D80" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{225097DF-B6D0-4122-AE89-AA7BA7CAC9B3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="23220" windowHeight="12390" tabRatio="590" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="23280" windowHeight="12480" tabRatio="590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
@@ -1793,27 +1793,27 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="3" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2352,106 +2352,106 @@
         <f ca="1">SUM(J11:X11,Y12:BQ12)</f>
         <v>-15621.779999999962</v>
       </c>
-      <c r="H11" s="143" t="s">
+      <c r="H11" s="144" t="s">
         <v>16</v>
       </c>
-      <c r="I11" s="144"/>
-      <c r="J11" s="138">
+      <c r="I11" s="139"/>
+      <c r="J11" s="143">
         <f t="array" aca="1" ref="J11" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))+SUMIFS(N15:N25,M15:M25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(J15:J25)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="139"/>
-      <c r="L11" s="139"/>
-      <c r="M11" s="139"/>
-      <c r="N11" s="140"/>
-      <c r="O11" s="138">
+      <c r="K11" s="141"/>
+      <c r="L11" s="141"/>
+      <c r="M11" s="141"/>
+      <c r="N11" s="142"/>
+      <c r="O11" s="143">
         <f t="array" aca="1" ref="O11" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))+SUMIFS(S15:S25,R15:R25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(O15:O25)</f>
         <v>81595.28</v>
       </c>
-      <c r="P11" s="139"/>
-      <c r="Q11" s="139"/>
-      <c r="R11" s="139"/>
-      <c r="S11" s="140"/>
-      <c r="T11" s="138">
+      <c r="P11" s="141"/>
+      <c r="Q11" s="141"/>
+      <c r="R11" s="141"/>
+      <c r="S11" s="142"/>
+      <c r="T11" s="143">
         <f t="array" aca="1" ref="T11" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))+SUMIFS(X15:X25,W15:W25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(T15:T25)</f>
         <v>46818.44</v>
       </c>
-      <c r="U11" s="139"/>
-      <c r="V11" s="139"/>
-      <c r="W11" s="139"/>
-      <c r="X11" s="140"/>
-      <c r="Y11" s="138">
+      <c r="U11" s="141"/>
+      <c r="V11" s="141"/>
+      <c r="W11" s="141"/>
+      <c r="X11" s="142"/>
+      <c r="Y11" s="143">
         <f t="array" aca="1" ref="Y11" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))+SUMIFS(AC15:AC25,AB15:AB25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(Y15:Y25)</f>
         <v>-54655.164444444439</v>
       </c>
-      <c r="Z11" s="139"/>
-      <c r="AA11" s="139"/>
-      <c r="AB11" s="139"/>
-      <c r="AC11" s="140"/>
-      <c r="AD11" s="138">
+      <c r="Z11" s="141"/>
+      <c r="AA11" s="141"/>
+      <c r="AB11" s="141"/>
+      <c r="AC11" s="142"/>
+      <c r="AD11" s="143">
         <f t="array" aca="1" ref="AD11" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))+SUMIFS(AH15:AH25,AG15:AG25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AD15:AD25)</f>
         <v>-9477.6644444444391</v>
       </c>
-      <c r="AE11" s="139"/>
-      <c r="AF11" s="139"/>
-      <c r="AG11" s="139"/>
-      <c r="AH11" s="140"/>
-      <c r="AI11" s="138">
+      <c r="AE11" s="141"/>
+      <c r="AF11" s="141"/>
+      <c r="AG11" s="141"/>
+      <c r="AH11" s="142"/>
+      <c r="AI11" s="143">
         <f t="array" aca="1" ref="AI11" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))+SUMIFS(AM15:AM25,AL15:AL25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AI15:AI25)</f>
         <v>-52174.224444444437</v>
       </c>
-      <c r="AJ11" s="139"/>
-      <c r="AK11" s="139"/>
-      <c r="AL11" s="139"/>
-      <c r="AM11" s="140"/>
-      <c r="AN11" s="138">
+      <c r="AJ11" s="141"/>
+      <c r="AK11" s="141"/>
+      <c r="AL11" s="141"/>
+      <c r="AM11" s="142"/>
+      <c r="AN11" s="143">
         <f t="array" aca="1" ref="AN11" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))+SUMIFS(AR15:AR25,AQ15:AQ25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AN15:AN25)</f>
         <v>-94366.444444444438</v>
       </c>
-      <c r="AO11" s="139"/>
-      <c r="AP11" s="139"/>
-      <c r="AQ11" s="139"/>
-      <c r="AR11" s="140"/>
-      <c r="AS11" s="138">
+      <c r="AO11" s="141"/>
+      <c r="AP11" s="141"/>
+      <c r="AQ11" s="141"/>
+      <c r="AR11" s="142"/>
+      <c r="AS11" s="143">
         <f t="array" aca="1" ref="AS11" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))+SUMIFS(AW15:AW25,AV15:AV25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AS15:AS25)</f>
         <v>-99787.444444444438</v>
       </c>
-      <c r="AT11" s="139"/>
-      <c r="AU11" s="139"/>
-      <c r="AV11" s="139"/>
-      <c r="AW11" s="140"/>
-      <c r="AX11" s="138">
+      <c r="AT11" s="141"/>
+      <c r="AU11" s="141"/>
+      <c r="AV11" s="141"/>
+      <c r="AW11" s="142"/>
+      <c r="AX11" s="143">
         <f t="array" aca="1" ref="AX11" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))+SUMIFS(BB15:BB25,BA15:BA25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(AX15:AX25)</f>
         <v>18688.055555555555</v>
       </c>
-      <c r="AY11" s="139"/>
-      <c r="AZ11" s="139"/>
-      <c r="BA11" s="139"/>
-      <c r="BB11" s="140"/>
-      <c r="BC11" s="138">
+      <c r="AY11" s="141"/>
+      <c r="AZ11" s="141"/>
+      <c r="BA11" s="141"/>
+      <c r="BB11" s="142"/>
+      <c r="BC11" s="143">
         <f t="array" aca="1" ref="BC11" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))+SUMIFS(BG15:BG25,BF15:BF25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BC15:BC25)</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BD11" s="139"/>
-      <c r="BE11" s="139"/>
-      <c r="BF11" s="139"/>
-      <c r="BG11" s="140"/>
-      <c r="BH11" s="138">
+      <c r="BD11" s="141"/>
+      <c r="BE11" s="141"/>
+      <c r="BF11" s="141"/>
+      <c r="BG11" s="142"/>
+      <c r="BH11" s="143">
         <f t="array" aca="1" ref="BH11" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))+SUMIFS(BL15:BL25,BK15:BK25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BH15:BH25)</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BI11" s="139"/>
-      <c r="BJ11" s="139"/>
-      <c r="BK11" s="139"/>
-      <c r="BL11" s="140"/>
-      <c r="BM11" s="138">
+      <c r="BI11" s="141"/>
+      <c r="BJ11" s="141"/>
+      <c r="BK11" s="141"/>
+      <c r="BL11" s="142"/>
+      <c r="BM11" s="143">
         <f t="array" aca="1" ref="BM11" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))+SUMIFS(BQ15:BQ25,BP15:BP25,"&lt;&gt;"&amp;"",$L$15:$L$25,"&lt;&gt;"&amp;"")+SUM(BM15:BM25)</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BN11" s="139"/>
-      <c r="BO11" s="139"/>
-      <c r="BP11" s="139"/>
-      <c r="BQ11" s="140"/>
+      <c r="BN11" s="141"/>
+      <c r="BO11" s="141"/>
+      <c r="BP11" s="141"/>
+      <c r="BQ11" s="142"/>
       <c r="BR11" s="21" t="s">
         <v>17</v>
       </c>
@@ -2483,106 +2483,106 @@
         <f ca="1">G11-G10</f>
         <v>-15621.779999999962</v>
       </c>
-      <c r="H12" s="147" t="s">
+      <c r="H12" s="138" t="s">
         <v>20</v>
       </c>
-      <c r="I12" s="144"/>
-      <c r="J12" s="138">
+      <c r="I12" s="139"/>
+      <c r="J12" s="143">
         <f t="array" aca="1" ref="J12" ca="1">SUM(M15:M25)+SUM(_xlfn._xlws.FILTER(L15:L25,M15:M25=""))+SUM(_xlfn._xlws.FILTER(K15:K25,(L15:L25="")*(M15:M25="")))</f>
         <v>47862.5</v>
       </c>
-      <c r="K12" s="139"/>
-      <c r="L12" s="139"/>
-      <c r="M12" s="139"/>
-      <c r="N12" s="140"/>
-      <c r="O12" s="138">
+      <c r="K12" s="141"/>
+      <c r="L12" s="141"/>
+      <c r="M12" s="141"/>
+      <c r="N12" s="142"/>
+      <c r="O12" s="143">
         <f t="array" aca="1" ref="O12" ca="1">SUM(R15:R25)+SUM(_xlfn._xlws.FILTER(Q15:Q25,R15:R25=""))+SUM(_xlfn._xlws.FILTER(P15:P25,(Q15:Q25="")*(R15:R25="")))</f>
         <v>17100</v>
       </c>
-      <c r="P12" s="139"/>
-      <c r="Q12" s="139"/>
-      <c r="R12" s="139"/>
-      <c r="S12" s="140"/>
-      <c r="T12" s="138">
+      <c r="P12" s="141"/>
+      <c r="Q12" s="141"/>
+      <c r="R12" s="141"/>
+      <c r="S12" s="142"/>
+      <c r="T12" s="143">
         <f t="array" aca="1" ref="T12" ca="1">SUM(W15:W25)+SUM(_xlfn._xlws.FILTER(V15:V25,W15:W25=""))+SUM(_xlfn._xlws.FILTER(U15:U25,(V15:V25="")*(W15:W25="")))</f>
         <v>79073</v>
       </c>
-      <c r="U12" s="139"/>
-      <c r="V12" s="139"/>
-      <c r="W12" s="139"/>
-      <c r="X12" s="140"/>
-      <c r="Y12" s="138">
+      <c r="U12" s="141"/>
+      <c r="V12" s="141"/>
+      <c r="W12" s="141"/>
+      <c r="X12" s="142"/>
+      <c r="Y12" s="143">
         <f t="array" aca="1" ref="Y12" ca="1">SUM(AB15:AB25)+SUM(_xlfn._xlws.FILTER(AA15:AA25,AB15:AB25=""))+SUM(_xlfn._xlws.FILTER(Z15:Z25,(AA15:AA25="")*(AB15:AB25="")))</f>
         <v>-2928.4444444444453</v>
       </c>
-      <c r="Z12" s="139"/>
-      <c r="AA12" s="139"/>
-      <c r="AB12" s="139"/>
-      <c r="AC12" s="140"/>
-      <c r="AD12" s="138">
+      <c r="Z12" s="141"/>
+      <c r="AA12" s="141"/>
+      <c r="AB12" s="141"/>
+      <c r="AC12" s="142"/>
+      <c r="AD12" s="143">
         <f t="array" aca="1" ref="AD12" ca="1">SUM(AG15:AG25)+SUM(_xlfn._xlws.FILTER(AF15:AF25,AG15:AG25=""))+SUM(_xlfn._xlws.FILTER(AE15:AE25,(AF15:AF25="")*(AG15:AG25="")))</f>
         <v>74786.555555555562</v>
       </c>
-      <c r="AE12" s="139"/>
-      <c r="AF12" s="139"/>
-      <c r="AG12" s="139"/>
-      <c r="AH12" s="140"/>
-      <c r="AI12" s="138">
+      <c r="AE12" s="141"/>
+      <c r="AF12" s="141"/>
+      <c r="AG12" s="141"/>
+      <c r="AH12" s="142"/>
+      <c r="AI12" s="143">
         <f t="array" aca="1" ref="AI12" ca="1">SUM(AL15:AL25)+SUM(_xlfn._xlws.FILTER(AK15:AK25,AL15:AL25=""))+SUM(_xlfn._xlws.FILTER(AJ15:AJ25,(AK15:AK25="")*(AL15:AL25="")))</f>
         <v>16094.555555555555</v>
       </c>
-      <c r="AJ12" s="139"/>
-      <c r="AK12" s="139"/>
-      <c r="AL12" s="139"/>
-      <c r="AM12" s="140"/>
-      <c r="AN12" s="138">
+      <c r="AJ12" s="141"/>
+      <c r="AK12" s="141"/>
+      <c r="AL12" s="141"/>
+      <c r="AM12" s="142"/>
+      <c r="AN12" s="143">
         <f t="array" aca="1" ref="AN12" ca="1">SUM(AQ15:AQ25)+SUM(_xlfn._xlws.FILTER(AP15:AP25,AQ15:AQ25=""))+SUM(_xlfn._xlws.FILTER(AO15:AO25,(AP15:AP25="")*(AQ15:AQ25="")))</f>
         <v>-38708.444444444445</v>
       </c>
-      <c r="AO12" s="139"/>
-      <c r="AP12" s="139"/>
-      <c r="AQ12" s="139"/>
-      <c r="AR12" s="140"/>
-      <c r="AS12" s="138">
+      <c r="AO12" s="141"/>
+      <c r="AP12" s="141"/>
+      <c r="AQ12" s="141"/>
+      <c r="AR12" s="142"/>
+      <c r="AS12" s="143">
         <f t="array" aca="1" ref="AS12" ca="1">SUM(AV15:AV25)+SUM(_xlfn._xlws.FILTER(AU15:AU25,AV15:AV25=""))+SUM(_xlfn._xlws.FILTER(AT15:AT25,(AU15:AU25="")*(AV15:AV25="")))</f>
         <v>-36735.944444444445</v>
       </c>
-      <c r="AT12" s="139"/>
-      <c r="AU12" s="139"/>
-      <c r="AV12" s="139"/>
-      <c r="AW12" s="140"/>
-      <c r="AX12" s="138">
+      <c r="AT12" s="141"/>
+      <c r="AU12" s="141"/>
+      <c r="AV12" s="141"/>
+      <c r="AW12" s="142"/>
+      <c r="AX12" s="143">
         <f t="array" aca="1" ref="AX12" ca="1">SUM(BA15:BA25)+SUM(_xlfn._xlws.FILTER(AZ15:AZ25,BA15:BA25=""))+SUM(_xlfn._xlws.FILTER(AY15:AY25,(AZ15:AZ25="")*(BA15:BA25="")))</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="AY12" s="139"/>
-      <c r="AZ12" s="139"/>
-      <c r="BA12" s="139"/>
-      <c r="BB12" s="140"/>
-      <c r="BC12" s="138">
+      <c r="AY12" s="141"/>
+      <c r="AZ12" s="141"/>
+      <c r="BA12" s="141"/>
+      <c r="BB12" s="142"/>
+      <c r="BC12" s="143">
         <f t="array" aca="1" ref="BC12" ca="1">SUM(BF15:BF25)+SUM(_xlfn._xlws.FILTER(BE15:BE25,BF15:BF25=""))+SUM(_xlfn._xlws.FILTER(BD15:BD25,(BE15:BE25="")*(BF15:BF25="")))</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BD12" s="139"/>
-      <c r="BE12" s="139"/>
-      <c r="BF12" s="139"/>
-      <c r="BG12" s="140"/>
-      <c r="BH12" s="138">
+      <c r="BD12" s="141"/>
+      <c r="BE12" s="141"/>
+      <c r="BF12" s="141"/>
+      <c r="BG12" s="142"/>
+      <c r="BH12" s="143">
         <f t="array" aca="1" ref="BH12" ca="1">SUM(BK15:BK25)+SUM(_xlfn._xlws.FILTER(BJ15:BJ25,BK15:BK25=""))+SUM(_xlfn._xlws.FILTER(BI15:BI25,(BJ15:BJ25="")*(BK15:BK25="")))</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BI12" s="139"/>
-      <c r="BJ12" s="139"/>
-      <c r="BK12" s="139"/>
-      <c r="BL12" s="140"/>
-      <c r="BM12" s="138">
+      <c r="BI12" s="141"/>
+      <c r="BJ12" s="141"/>
+      <c r="BK12" s="141"/>
+      <c r="BL12" s="142"/>
+      <c r="BM12" s="143">
         <f t="array" aca="1" ref="BM12" ca="1">SUM(BP15:BP25)+SUM(_xlfn._xlws.FILTER(BO15:BO25,BP15:BP25=""))+SUM(_xlfn._xlws.FILTER(BN15:BN25,(BO15:BO25="")*(BP15:BP25="")))</f>
         <v>-39135.944444444445</v>
       </c>
-      <c r="BN12" s="139"/>
-      <c r="BO12" s="139"/>
-      <c r="BP12" s="139"/>
-      <c r="BQ12" s="140"/>
+      <c r="BN12" s="141"/>
+      <c r="BO12" s="141"/>
+      <c r="BP12" s="141"/>
+      <c r="BQ12" s="142"/>
       <c r="BR12" s="21"/>
       <c r="BS12" s="22"/>
     </row>
@@ -2594,90 +2594,90 @@
         <v>22</v>
       </c>
       <c r="I13" s="146"/>
-      <c r="J13" s="142">
+      <c r="J13" s="147">
         <v>45688</v>
       </c>
-      <c r="K13" s="139"/>
-      <c r="L13" s="139"/>
-      <c r="M13" s="139"/>
-      <c r="N13" s="139"/>
-      <c r="O13" s="141" t="s">
+      <c r="K13" s="141"/>
+      <c r="L13" s="141"/>
+      <c r="M13" s="141"/>
+      <c r="N13" s="141"/>
+      <c r="O13" s="140" t="s">
         <v>23</v>
       </c>
-      <c r="P13" s="139"/>
-      <c r="Q13" s="139"/>
-      <c r="R13" s="139"/>
-      <c r="S13" s="140"/>
-      <c r="T13" s="141">
+      <c r="P13" s="141"/>
+      <c r="Q13" s="141"/>
+      <c r="R13" s="141"/>
+      <c r="S13" s="142"/>
+      <c r="T13" s="140">
         <v>45747</v>
       </c>
-      <c r="U13" s="139"/>
-      <c r="V13" s="139"/>
-      <c r="W13" s="139"/>
-      <c r="X13" s="140"/>
-      <c r="Y13" s="141">
+      <c r="U13" s="141"/>
+      <c r="V13" s="141"/>
+      <c r="W13" s="141"/>
+      <c r="X13" s="142"/>
+      <c r="Y13" s="140">
         <v>45777</v>
       </c>
-      <c r="Z13" s="139"/>
-      <c r="AA13" s="139"/>
-      <c r="AB13" s="139"/>
-      <c r="AC13" s="140"/>
-      <c r="AD13" s="141">
+      <c r="Z13" s="141"/>
+      <c r="AA13" s="141"/>
+      <c r="AB13" s="141"/>
+      <c r="AC13" s="142"/>
+      <c r="AD13" s="140">
         <v>45808</v>
       </c>
-      <c r="AE13" s="139"/>
-      <c r="AF13" s="139"/>
-      <c r="AG13" s="139"/>
-      <c r="AH13" s="140"/>
-      <c r="AI13" s="141">
+      <c r="AE13" s="141"/>
+      <c r="AF13" s="141"/>
+      <c r="AG13" s="141"/>
+      <c r="AH13" s="142"/>
+      <c r="AI13" s="140">
         <v>45838</v>
       </c>
-      <c r="AJ13" s="139"/>
-      <c r="AK13" s="139"/>
-      <c r="AL13" s="139"/>
-      <c r="AM13" s="140"/>
-      <c r="AN13" s="141">
+      <c r="AJ13" s="141"/>
+      <c r="AK13" s="141"/>
+      <c r="AL13" s="141"/>
+      <c r="AM13" s="142"/>
+      <c r="AN13" s="140">
         <v>45869</v>
       </c>
-      <c r="AO13" s="139"/>
-      <c r="AP13" s="139"/>
-      <c r="AQ13" s="139"/>
-      <c r="AR13" s="140"/>
-      <c r="AS13" s="141">
+      <c r="AO13" s="141"/>
+      <c r="AP13" s="141"/>
+      <c r="AQ13" s="141"/>
+      <c r="AR13" s="142"/>
+      <c r="AS13" s="140">
         <v>45900</v>
       </c>
-      <c r="AT13" s="139"/>
-      <c r="AU13" s="139"/>
-      <c r="AV13" s="139"/>
-      <c r="AW13" s="140"/>
-      <c r="AX13" s="141">
+      <c r="AT13" s="141"/>
+      <c r="AU13" s="141"/>
+      <c r="AV13" s="141"/>
+      <c r="AW13" s="142"/>
+      <c r="AX13" s="140">
         <v>45930</v>
       </c>
-      <c r="AY13" s="139"/>
-      <c r="AZ13" s="139"/>
-      <c r="BA13" s="139"/>
-      <c r="BB13" s="140"/>
-      <c r="BC13" s="141">
+      <c r="AY13" s="141"/>
+      <c r="AZ13" s="141"/>
+      <c r="BA13" s="141"/>
+      <c r="BB13" s="142"/>
+      <c r="BC13" s="140">
         <v>45961</v>
       </c>
-      <c r="BD13" s="139"/>
-      <c r="BE13" s="139"/>
-      <c r="BF13" s="139"/>
-      <c r="BG13" s="140"/>
-      <c r="BH13" s="141">
+      <c r="BD13" s="141"/>
+      <c r="BE13" s="141"/>
+      <c r="BF13" s="141"/>
+      <c r="BG13" s="142"/>
+      <c r="BH13" s="140">
         <v>45991</v>
       </c>
-      <c r="BI13" s="139"/>
-      <c r="BJ13" s="139"/>
-      <c r="BK13" s="139"/>
-      <c r="BL13" s="140"/>
-      <c r="BM13" s="141">
+      <c r="BI13" s="141"/>
+      <c r="BJ13" s="141"/>
+      <c r="BK13" s="141"/>
+      <c r="BL13" s="142"/>
+      <c r="BM13" s="140">
         <v>46022</v>
       </c>
-      <c r="BN13" s="139"/>
-      <c r="BO13" s="139"/>
-      <c r="BP13" s="139"/>
-      <c r="BQ13" s="140"/>
+      <c r="BN13" s="141"/>
+      <c r="BO13" s="141"/>
+      <c r="BP13" s="141"/>
+      <c r="BQ13" s="142"/>
       <c r="BR13" s="24">
         <f>SUM(BR15:BR24)</f>
         <v>352223.5</v>
@@ -4358,13 +4358,20 @@
   </sheetData>
   <autoFilter ref="B14:B20" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="39">
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="AS13:AW13"/>
-    <mergeCell ref="BC13:BG13"/>
-    <mergeCell ref="Y12:AC12"/>
-    <mergeCell ref="AI12:AM12"/>
-    <mergeCell ref="J12:N12"/>
-    <mergeCell ref="AN13:AR13"/>
+    <mergeCell ref="BM12:BQ12"/>
+    <mergeCell ref="BC11:BG11"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="BM11:BQ11"/>
+    <mergeCell ref="AD13:AH13"/>
+    <mergeCell ref="Y11:AC11"/>
+    <mergeCell ref="BH12:BL12"/>
+    <mergeCell ref="AX11:BB11"/>
+    <mergeCell ref="AS12:AW12"/>
+    <mergeCell ref="AI11:AM11"/>
+    <mergeCell ref="BM13:BQ13"/>
+    <mergeCell ref="BH13:BL13"/>
+    <mergeCell ref="O11:S11"/>
+    <mergeCell ref="BH11:BL11"/>
     <mergeCell ref="H11:I11"/>
     <mergeCell ref="T12:X12"/>
     <mergeCell ref="J11:N11"/>
@@ -4381,22 +4388,15 @@
     <mergeCell ref="O13:S13"/>
     <mergeCell ref="T13:X13"/>
     <mergeCell ref="O12:S12"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="AS13:AW13"/>
+    <mergeCell ref="BC13:BG13"/>
+    <mergeCell ref="Y12:AC12"/>
+    <mergeCell ref="AI12:AM12"/>
+    <mergeCell ref="J12:N12"/>
+    <mergeCell ref="AN13:AR13"/>
     <mergeCell ref="AD12:AH12"/>
     <mergeCell ref="AI13:AM13"/>
-    <mergeCell ref="BM12:BQ12"/>
-    <mergeCell ref="BC11:BG11"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="BM11:BQ11"/>
-    <mergeCell ref="AD13:AH13"/>
-    <mergeCell ref="Y11:AC11"/>
-    <mergeCell ref="BH12:BL12"/>
-    <mergeCell ref="AX11:BB11"/>
-    <mergeCell ref="AS12:AW12"/>
-    <mergeCell ref="AI11:AM11"/>
-    <mergeCell ref="BM13:BQ13"/>
-    <mergeCell ref="BH13:BL13"/>
-    <mergeCell ref="O11:S11"/>
-    <mergeCell ref="BH11:BL11"/>
   </mergeCells>
   <conditionalFormatting sqref="M15:M24 R15:R24 W15:W24 AB15:AB24 AG15:AG24 AL15:AL24 AQ15:AQ24 AV15:AV24 BA15:BA24 BF15:BF24 BK15:BK24 BP15:BP24">
     <cfRule type="expression" dxfId="7" priority="8">
@@ -5222,7 +5222,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="2" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>85</v>
       </c>
@@ -5502,7 +5502,7 @@
         <v>34040</v>
       </c>
     </row>
-    <row r="4" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>85</v>
       </c>
@@ -5782,7 +5782,7 @@
         <v>62210</v>
       </c>
     </row>
-    <row r="6" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -6062,7 +6062,7 @@
         <v>58648</v>
       </c>
     </row>
-    <row r="8" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>85</v>
       </c>
@@ -6762,7 +6762,7 @@
         <v>-18462</v>
       </c>
     </row>
-    <row r="13" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>85</v>
       </c>
@@ -6902,7 +6902,7 @@
         <v>-22813.72</v>
       </c>
     </row>
-    <row r="14" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>85</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>19294.5</v>
       </c>
     </row>
-    <row r="15" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>85</v>
       </c>
@@ -7742,7 +7742,7 @@
         <v>18112</v>
       </c>
     </row>
-    <row r="20" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>85</v>
       </c>
@@ -8582,7 +8582,7 @@
         <v>20960</v>
       </c>
     </row>
-    <row r="26" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>85</v>
       </c>
@@ -9282,7 +9282,7 @@
         <v>-18502</v>
       </c>
     </row>
-    <row r="31" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>85</v>
       </c>
@@ -9422,7 +9422,7 @@
         <v>-19294.5</v>
       </c>
     </row>
-    <row r="32" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -10122,7 +10122,7 @@
         <v>48000</v>
       </c>
     </row>
-    <row r="37" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>85</v>
       </c>
@@ -10682,7 +10682,7 @@
         <v>98592</v>
       </c>
     </row>
-    <row r="41" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>85</v>
       </c>
@@ -10822,7 +10822,7 @@
         <v>-20952.78</v>
       </c>
     </row>
-    <row r="42" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>85</v>
       </c>
@@ -11242,7 +11242,7 @@
         <v>57824</v>
       </c>
     </row>
-    <row r="45" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>85</v>
       </c>
@@ -11382,7 +11382,7 @@
         <v>-13632.5</v>
       </c>
     </row>
-    <row r="46" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -11522,7 +11522,7 @@
         <v>13632.5</v>
       </c>
     </row>
-    <row r="47" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>85</v>
       </c>
@@ -11802,7 +11802,7 @@
         <v>-60224</v>
       </c>
     </row>
-    <row r="49" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>85</v>
       </c>
@@ -11942,7 +11942,7 @@
         <v>-14060</v>
       </c>
     </row>
-    <row r="50" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>85</v>
       </c>
@@ -12222,7 +12222,7 @@
         <v>38368</v>
       </c>
     </row>
-    <row r="52" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>85</v>
       </c>
@@ -12642,7 +12642,7 @@
         <v>60224</v>
       </c>
     </row>
-    <row r="55" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>85</v>
       </c>
@@ -12782,7 +12782,7 @@
         <v>-30922.5</v>
       </c>
     </row>
-    <row r="56" spans="1:47" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:47" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>85</v>
       </c>
@@ -12924,9 +12924,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L56" xr:uid="{00000000-0009-0000-0000-000002000000}">
-    <filterColumn colId="11">
+    <filterColumn colId="0">
       <filters>
-        <filter val="Reclass"/>
+        <filter val="9500879389"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>